<commit_message>
Update firm list spreadsheet and remove thumbnail
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/All_CA_firm_list_in_bangladesh- execl file.xlsx
+++ b/All_CA_firm_list_in_bangladesh- execl file.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\COMPUTER CITY\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Download 2\MY all Projects\RoadToCA website\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A4F0C1A7-9F4E-4597-B8C6-834ACA6C5F37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{165E8342-3990-42E1-992E-41FD1340D8BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="CA Firms Bangladesh Directory" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -1719,6 +1718,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:H262"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -8493,6 +8495,6 @@
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup scale="45" fitToWidth="0" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup scale="45" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>